<commit_message>
v5.12 scan 2026-09-14 05:46 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14382,14 +14382,14 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-111.69</v>
+        <v>-109.5</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P5" s="11" t="inlineStr">
         <is>
-          <t>~-122.15 (unrealized)</t>
+          <t>~-119.96 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="11" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 16:21 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>6.8</v>
+        <v>10.21</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P2" s="10" t="inlineStr">
         <is>
-          <t>~-3.38 (unrealized)</t>
+          <t>~0.03 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="10" t="inlineStr">
         <is>
-          <t>~+0.20%</t>
+          <t>~+0.30%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-109.5</v>
+        <v>-429.97</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>~-119.96 (unrealized)</t>
+          <t>~-440.43 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
         <is>
-          <t>~-0.21%</t>
+          <t>~-0.82%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-389.36</v>
+        <v>401.92</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>~-399.82 (unrealized)</t>
+          <t>~391.46 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="10" t="inlineStr">
         <is>
-          <t>~-0.74%</t>
+          <t>~+0.77%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 18:09 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>10.21</v>
+        <v>13.25</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P2" s="10" t="inlineStr">
         <is>
-          <t>~0.03 (unrealized)</t>
+          <t>~3.07 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="10" t="inlineStr">
         <is>
-          <t>~+0.30%</t>
+          <t>~+0.39%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-429.97</v>
+        <v>-289.81</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>~-440.43 (unrealized)</t>
+          <t>~-300.27 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
         <is>
-          <t>~-0.82%</t>
+          <t>~-0.55%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>401.92</v>
+        <v>320.28</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>~391.46 (unrealized)</t>
+          <t>~309.82 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="10" t="inlineStr">
         <is>
-          <t>~+0.77%</t>
+          <t>~+0.61%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 19:33 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-127.41</v>
+        <v>-158.92</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-137.83 (unrealized)</t>
+          <t>~-169.34 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.24%</t>
+          <t>~-0.30%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>1097.43</v>
+        <v>1144.08</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~1,086.93 (unrealized)</t>
+          <t>~1,133.58 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+2.09%</t>
+          <t>~+2.18%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>733.59</v>
+        <v>724.1799999999999</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~723.13 (unrealized)</t>
+          <t>~713.72 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+1.40%</t>
+          <t>~+1.39%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>13.3</v>
+        <v>10.68</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~3.12 (unrealized)</t>
+          <t>~0.50 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+0.39%</t>
+          <t>~+0.31%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-319.74</v>
+        <v>-382.52</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-330.20 (unrealized)</t>
+          <t>~-392.98 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-0.61%</t>
+          <t>~-0.73%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>348.54</v>
+        <v>395.67</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~338.08 (unrealized)</t>
+          <t>~385.21 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.67%</t>
+          <t>~+0.76%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 19:53 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-158.92</v>
+        <v>-184.26</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-169.34 (unrealized)</t>
+          <t>~-194.68 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.30%</t>
+          <t>~-0.35%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,14 +14182,14 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>1144.08</v>
+        <v>1141.7</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~1,133.58 (unrealized)</t>
+          <t>~1,131.20 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>724.1799999999999</v>
+        <v>667.76</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~713.72 (unrealized)</t>
+          <t>~657.30 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+1.39%</t>
+          <t>~+1.28%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>10.68</v>
+        <v>11.18</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~0.50 (unrealized)</t>
+          <t>~1.00 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+0.31%</t>
+          <t>~+0.33%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-382.52</v>
+        <v>-448.22</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-392.98 (unrealized)</t>
+          <t>~-458.68 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-0.73%</t>
+          <t>~-0.86%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>395.67</v>
+        <v>329.7</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~385.21 (unrealized)</t>
+          <t>~319.24 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.76%</t>
+          <t>~+0.63%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 20:23 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-184.26</v>
+        <v>-220.57</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-194.68 (unrealized)</t>
+          <t>~-230.99 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.35%</t>
+          <t>~-0.42%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,14 +14182,14 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>1141.7</v>
+        <v>1146.36</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~1,131.20 (unrealized)</t>
+          <t>~1,135.86 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>667.76</v>
+        <v>645.8099999999999</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~657.30 (unrealized)</t>
+          <t>~635.35 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+1.28%</t>
+          <t>~+1.24%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>11.18</v>
+        <v>14.84</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~1.00 (unrealized)</t>
+          <t>~4.66 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+0.33%</t>
+          <t>~+0.44%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-448.22</v>
+        <v>-527.0599999999999</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-458.68 (unrealized)</t>
+          <t>~-537.52 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-0.86%</t>
+          <t>~-1.01%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>329.7</v>
+        <v>361.1</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~319.24 (unrealized)</t>
+          <t>~350.64 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.63%</t>
+          <t>~+0.69%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 21:44 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>14.84</v>
+        <v>-1.04</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~4.66 (unrealized)</t>
+          <t>~-11.22 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+0.44%</t>
+          <t>~-0.03%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 22:36 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-1.04</v>
+        <v>-6.44</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-11.22 (unrealized)</t>
+          <t>~-16.62 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-0.03%</t>
+          <t>~-0.19%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-14 23:21 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-6.44</v>
+        <v>-8.789999999999999</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-16.62 (unrealized)</t>
+          <t>~-18.97 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-0.19%</t>
+          <t>~-0.26%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 06:01 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-8.789999999999999</v>
+        <v>-16.67</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-18.97 (unrealized)</t>
+          <t>~-26.85 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-0.26%</t>
+          <t>~-0.49%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 09:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-16.67</v>
+        <v>-15.64</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-26.85 (unrealized)</t>
+          <t>~-25.82 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-0.49%</t>
+          <t>~-0.46%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 14:59 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-220.57</v>
+        <v>-605.54</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-230.99 (unrealized)</t>
+          <t>~-615.96 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.42%</t>
+          <t>~-1.16%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>1146.36</v>
+        <v>608.13</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~1,135.86 (unrealized)</t>
+          <t>~597.63 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+2.18%</t>
+          <t>~+1.16%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>645.8099999999999</v>
+        <v>316.63</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~635.35 (unrealized)</t>
+          <t>~306.17 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+1.24%</t>
+          <t>~+0.61%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-15.64</v>
+        <v>-28.47</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-25.82 (unrealized)</t>
+          <t>~-38.65 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-0.46%</t>
+          <t>~-0.84%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-527.0599999999999</v>
+        <v>-858.85</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-537.52 (unrealized)</t>
+          <t>~-869.31 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.01%</t>
+          <t>~-1.64%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>361.1</v>
+        <v>106.76</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~350.64 (unrealized)</t>
+          <t>~96.30 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.69%</t>
+          <t>~+0.20%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 17:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-605.54</v>
+        <v>-595.95</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-615.96 (unrealized)</t>
+          <t>~-606.37 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-1.16%</t>
+          <t>~-1.14%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>608.13</v>
+        <v>734.1799999999999</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~597.63 (unrealized)</t>
+          <t>~723.68 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.16%</t>
+          <t>~+1.40%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>316.63</v>
+        <v>347.98</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~306.17 (unrealized)</t>
+          <t>~337.52 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.61%</t>
+          <t>~+0.67%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-28.47</v>
+        <v>-41.44</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-38.65 (unrealized)</t>
+          <t>~-51.62 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-0.84%</t>
+          <t>~-1.22%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-858.85</v>
+        <v>-816.87</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-869.31 (unrealized)</t>
+          <t>~-827.33 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.64%</t>
+          <t>~-1.56%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>106.76</v>
+        <v>392.5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~96.30 (unrealized)</t>
+          <t>~382.04 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.20%</t>
+          <t>~+0.75%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 17:44 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>734.1799999999999</v>
+        <v>729.29</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~723.68 (unrealized)</t>
+          <t>~718.79 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.40%</t>
+          <t>~+1.39%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-41.44</v>
+        <v>-48.37</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-51.62 (unrealized)</t>
+          <t>~-58.55 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.22%</t>
+          <t>~-1.43%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-816.87</v>
+        <v>-851.91</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-827.33 (unrealized)</t>
+          <t>~-862.37 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.56%</t>
+          <t>~-1.63%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>392.5</v>
+        <v>310.86</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~382.04 (unrealized)</t>
+          <t>~300.40 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.75%</t>
+          <t>~+0.59%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 18:24 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-595.95</v>
+        <v>-580.63</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-606.37 (unrealized)</t>
+          <t>~-591.05 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-1.14%</t>
+          <t>~-1.11%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>729.29</v>
+        <v>785.21</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~718.79 (unrealized)</t>
+          <t>~774.71 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.39%</t>
+          <t>~+1.50%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-48.37</v>
+        <v>-67.45</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-58.55 (unrealized)</t>
+          <t>~-77.63 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.43%</t>
+          <t>~-1.99%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-851.91</v>
+        <v>-819.79</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-862.37 (unrealized)</t>
+          <t>~-830.25 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.63%</t>
+          <t>~-1.57%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>310.86</v>
+        <v>351.68</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~300.40 (unrealized)</t>
+          <t>~341.22 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~+0.59%</t>
+          <t>~+0.67%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 19:08 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -1099,17 +1099,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>#14ID IWM SHORT</t>
+          <t>#4SW XLV LONG</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1119,46 +1119,46 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Price&lt;SMA50+EMA9&gt;EMA20+EMA20&lt;EMA50+Close&gt;Open</t>
+          <t>EMA9&gt;EMA20+Range&lt;1%</t>
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>63.41</v>
+        <v>52.32</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>7.5</v>
+        <v>23.85</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>1182.87</v>
+        <v>1420.63</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>19.75</v>
+        <v>61.23</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>1163.12</v>
+        <v>1359.4</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>1163.12</v>
+        <v>226.57</v>
       </c>
     </row>
     <row r="10">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>#36ID DIA LONG</t>
+          <t>#14ID IWM SHORT</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1187,46 +1187,46 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Price&lt;SMA50+EMA9&gt;EMA20+Close&lt;Open+2Red</t>
+          <t>Price&lt;SMA50+EMA9&gt;EMA20+EMA20&lt;EMA50+Close&gt;Open</t>
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>67.86</v>
+        <v>63.41</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2.52</v>
+        <v>7.5</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1221.22</v>
+        <v>1182.87</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>76.68000000000001</v>
+        <v>19.75</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>1144.54</v>
+        <v>1163.12</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>286.13</v>
+        <v>1163.12</v>
       </c>
     </row>
     <row r="11">
@@ -1235,17 +1235,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>#4SW XLV LONG</t>
+          <t>#36ID DIA LONG</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1260,41 +1260,41 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Range&lt;1%</t>
+          <t>Price&lt;SMA50+EMA9&gt;EMA20+Close&lt;Open+2Red</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>52.32</v>
+        <v>67.86</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>23.85</v>
+        <v>2.52</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>2</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>1137.01</v>
+        <v>1221.22</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>50.77</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>1086.24</v>
+        <v>1144.54</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>217.25</v>
+        <v>286.13</v>
       </c>
     </row>
     <row r="12">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>#31SW QQQ LONG</t>
+          <t>#4SW XLP LONG</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2280,14 +2280,14 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+2Red</t>
+          <t>EMA20&lt;EMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>65.29000000000001</v>
+        <v>61.78</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>48.57</v>
+        <v>70.52</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1</v>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>#4SW XLP LONG</t>
+          <t>#1SW TRX-USD LONG</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2333,12 +2333,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>TRX-USD</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2348,41 +2348,41 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>EMA20&lt;EMA50+Range&lt;1%</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>61.78</v>
+        <v>66.67</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>70.52</v>
+        <v>51.86</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>0</v>
+        <v>-27.64</v>
       </c>
       <c r="P27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>0</v>
+        <v>40.12</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>-67.76000000000001</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>0</v>
+        <v>-16.94</v>
       </c>
     </row>
     <row r="28">
@@ -2391,17 +2391,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>#1SW TRX-USD LONG</t>
+          <t>#1ID DOGE-USD SHORT</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>TRX-USD</t>
+          <t>DOGE-USD</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2411,46 +2411,46 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>66.67</v>
+        <v>50.67</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>51.86</v>
+        <v>31.42</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="N28" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>-27.64</v>
+        <v>-88.45</v>
       </c>
       <c r="P28" s="4" t="n">
-        <v>40.12</v>
+        <v>12.57</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>-67.76000000000001</v>
+        <v>-101.02</v>
       </c>
       <c r="R28" s="4" t="n">
-        <v>-16.94</v>
+        <v>-101.02</v>
       </c>
     </row>
     <row r="29">
@@ -2459,66 +2459,66 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>#1ID DOGE-USD SHORT</t>
+          <t>#5SW XLP LONG</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>DOGE-USD</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>Range&lt;1%+SMA20&lt;EMA20</t>
         </is>
       </c>
       <c r="H29" s="4" t="n">
-        <v>50.67</v>
+        <v>58.26</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>31.42</v>
+        <v>67.47</v>
       </c>
       <c r="J29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O29" s="4" t="n">
-        <v>-88.45</v>
+        <v>-149.74</v>
       </c>
       <c r="P29" s="4" t="n">
-        <v>12.57</v>
+        <v>20.27</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>-101.02</v>
+        <v>-170.01</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>-101.02</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="30">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>#5SW XLP LONG</t>
+          <t>#57SW XLRE LONG</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2552,41 +2552,41 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Range&lt;1%+SMA20&lt;EMA20</t>
+          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&lt;Open</t>
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>58.26</v>
+        <v>69.23</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>67.47</v>
+        <v>16.84</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O30" s="4" t="n">
-        <v>-149.74</v>
+        <v>-469.04</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>20.27</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>-170.01</v>
+        <v>-479</v>
       </c>
       <c r="R30" s="4" t="n">
-        <v>-85</v>
+        <v>-479</v>
       </c>
     </row>
     <row r="31">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>#57SW XLRE LONG</t>
+          <t>#3SW XLC LONG</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2620,20 +2620,20 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&lt;Open</t>
+          <t>Price&gt;EMA9+Range&lt;1%</t>
         </is>
       </c>
       <c r="H31" s="4" t="n">
-        <v>69.23</v>
+        <v>53.98</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>16.84</v>
+        <v>68.92</v>
       </c>
       <c r="J31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K31" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2645,16 +2645,16 @@
         <v>0</v>
       </c>
       <c r="O31" s="4" t="n">
-        <v>-469.04</v>
+        <v>-750.65</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>9.960000000000001</v>
+        <v>10.32</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>-479</v>
+        <v>-760.97</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>-479</v>
+        <v>-760.97</v>
       </c>
     </row>
     <row r="32">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>#3SW XLC LONG</t>
+          <t>#31SW QQQ LONG</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2688,20 +2688,20 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;EMA9+Range&lt;1%</t>
+          <t>Price&gt;SMA50+2Red</t>
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>53.98</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>68.92</v>
+        <v>48.57</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2713,16 +2713,16 @@
         <v>0</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-750.65</v>
+        <v>-865.8099999999999</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>10.32</v>
+        <v>10.46</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
       <c r="R32" s="4" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
     </row>
     <row r="33">
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-580.63</v>
+        <v>-572.66</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-591.05 (unrealized)</t>
+          <t>~-583.08 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-1.11%</t>
+          <t>~-1.10%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>785.21</v>
+        <v>745.6</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~774.71 (unrealized)</t>
+          <t>~735.10 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.50%</t>
+          <t>~+1.42%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>347.98</v>
+        <v>366.79</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~337.52 (unrealized)</t>
+          <t>~356.33 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.67%</t>
+          <t>~+0.70%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-67.45</v>
+        <v>-68.56999999999999</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-77.63 (unrealized)</t>
+          <t>~-78.75 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.99%</t>
+          <t>~-2.02%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14767,27 +14767,29 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="L9" s="2" t="n">
+        <v>704.52</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:37:33 IST</t>
+        </is>
+      </c>
       <c r="N9" s="4" t="n">
-        <v>-819.79</v>
+        <v>-865.8099999999999</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
-      <c r="P9" s="9" t="inlineStr">
-        <is>
-          <t>~-830.25 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>~-1.57%</t>
-        </is>
+      <c r="P9" s="6" t="n">
+        <v>-876.27</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>-1.68</v>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -14812,7 +14814,7 @@
       </c>
       <c r="W9" s="3" t="inlineStr">
         <is>
-          <t>#31SW Price&gt;SMA50+2Red</t>
+          <t>#31SW Price&gt;SMA50+2Red | Expiry 5d</t>
         </is>
       </c>
     </row>
@@ -14864,27 +14866,29 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="L10" s="2" t="n">
+        <v>167.5</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:37:33 IST</t>
+        </is>
+      </c>
       <c r="N10" s="4" t="n">
-        <v>351.68</v>
+        <v>283.62</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.46</v>
       </c>
-      <c r="P10" s="9" t="inlineStr">
-        <is>
-          <t>~341.22 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>~+0.67%</t>
-        </is>
+      <c r="P10" s="5" t="n">
+        <v>273.16</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>0.52</v>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -14909,7 +14913,7 @@
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
-          <t>#4SW EMA9&gt;EMA20+Range&lt;1%</t>
+          <t>#4SW EMA9&gt;EMA20+Range&lt;1% | Expiry 5d</t>
         </is>
       </c>
     </row>
@@ -20547,18 +20551,18 @@
       <c r="L68" s="15" t="inlineStr"/>
       <c r="M68" s="14" t="inlineStr"/>
       <c r="N68" s="17" t="n">
-        <v>26493.04</v>
+        <v>25910.85</v>
       </c>
       <c r="O68" s="17" t="n">
-        <v>2438.67</v>
+        <v>2459.59</v>
       </c>
       <c r="P68" s="18" t="n">
-        <v>24054.37</v>
+        <v>23451.26</v>
       </c>
       <c r="Q68" s="16" t="inlineStr"/>
       <c r="R68" s="15" t="inlineStr">
         <is>
-          <t>66 trades (60 closed / 6 open)</t>
+          <t>66 trades (62 closed / 4 open)</t>
         </is>
       </c>
       <c r="S68" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 19:46 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-572.66</v>
+        <v>-628.83</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-583.08 (unrealized)</t>
+          <t>~-639.25 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-1.10%</t>
+          <t>~-1.21%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>745.6</v>
+        <v>605.8</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~735.10 (unrealized)</t>
+          <t>~595.30 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.42%</t>
+          <t>~+1.15%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>366.79</v>
+        <v>241.4</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~356.33 (unrealized)</t>
+          <t>~230.94 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.70%</t>
+          <t>~+0.46%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-68.56999999999999</v>
+        <v>-65.62</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-78.75 (unrealized)</t>
+          <t>~-75.80 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-2.02%</t>
+          <t>~-1.93%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 21:10 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-628.83</v>
+        <v>-557.59</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-639.25 (unrealized)</t>
+          <t>~-568.01 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-1.21%</t>
+          <t>~-1.07%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>605.8</v>
+        <v>661.72</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~595.30 (unrealized)</t>
+          <t>~651.22 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.15%</t>
+          <t>~+1.26%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>241.4</v>
+        <v>213.18</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~230.94 (unrealized)</t>
+          <t>~202.72 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.46%</t>
+          <t>~+0.41%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-65.62</v>
+        <v>-70.47</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-75.80 (unrealized)</t>
+          <t>~-80.65 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.93%</t>
+          <t>~-2.08%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 22:21 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-70.47</v>
+        <v>-68.98999999999999</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-80.65 (unrealized)</t>
+          <t>~-79.17 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-2.08%</t>
+          <t>~-2.03%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-15 23:06 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-68.98999999999999</v>
+        <v>-62.56</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-79.17 (unrealized)</t>
+          <t>~-72.74 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-2.03%</t>
+          <t>~-1.84%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 03:15 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-62.56</v>
+        <v>-64.42</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-72.74 (unrealized)</t>
+          <t>~-74.60 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.84%</t>
+          <t>~-1.90%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 05:51 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-64.42</v>
+        <v>-50.01</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-74.60 (unrealized)</t>
+          <t>~-60.19 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.90%</t>
+          <t>~-1.47%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 08:49 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-50.01</v>
+        <v>-45.93</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-60.19 (unrealized)</t>
+          <t>~-56.11 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.47%</t>
+          <t>~-1.35%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 09:05 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-45.93</v>
+        <v>-48.51</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-56.11 (unrealized)</t>
+          <t>~-58.69 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.35%</t>
+          <t>~-1.43%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 14:01 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-557.59</v>
+        <v>-346.61</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-568.01 (unrealized)</t>
+          <t>~-357.03 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-1.07%</t>
+          <t>~-0.67%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>661.72</v>
+        <v>801.52</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~651.22 (unrealized)</t>
+          <t>~791.02 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.26%</t>
+          <t>~+1.53%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,14 +14279,14 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>213.18</v>
+        <v>216.32</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~202.72 (unrealized)</t>
+          <t>~205.86 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-48.51</v>
+        <v>-47.97</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-58.69 (unrealized)</t>
+          <t>~-58.15 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.43%</t>
+          <t>~-1.41%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 14:56 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-346.61</v>
+        <v>-397.3</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-357.03 (unrealized)</t>
+          <t>~-407.72 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.67%</t>
+          <t>~-0.76%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>801.52</v>
+        <v>771.23</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~791.02 (unrealized)</t>
+          <t>~760.73 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.53%</t>
+          <t>~+1.47%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>216.32</v>
+        <v>225.72</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~205.86 (unrealized)</t>
+          <t>~215.26 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.41%</t>
+          <t>~+0.43%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-47.97</v>
+        <v>-47.11</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-58.15 (unrealized)</t>
+          <t>~-57.29 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.41%</t>
+          <t>~-1.39%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 17:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-397.3</v>
+        <v>-426.07</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-407.72 (unrealized)</t>
+          <t>~-436.49 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.76%</t>
+          <t>~-0.82%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>771.23</v>
+        <v>652.4</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~760.73 (unrealized)</t>
+          <t>~641.90 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.47%</t>
+          <t>~+1.24%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>225.72</v>
+        <v>319.77</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~215.26 (unrealized)</t>
+          <t>~309.31 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.43%</t>
+          <t>~+0.61%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-47.11</v>
+        <v>-36.68</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-57.29 (unrealized)</t>
+          <t>~-46.86 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.39%</t>
+          <t>~-1.08%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 17:42 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-426.07</v>
+        <v>-430.18</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-436.49 (unrealized)</t>
+          <t>~-440.60 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.82%</t>
+          <t>~-0.83%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>652.4</v>
+        <v>570.85</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~641.90 (unrealized)</t>
+          <t>~560.35 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.24%</t>
+          <t>~+1.09%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>319.77</v>
+        <v>363.72</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~309.31 (unrealized)</t>
+          <t>~353.26 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.61%</t>
+          <t>~+0.70%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-36.68</v>
+        <v>-37.57</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-46.86 (unrealized)</t>
+          <t>~-47.75 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.08%</t>
+          <t>~-1.11%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 18:20 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>-430.18</v>
+        <v>-387.7</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-440.60 (unrealized)</t>
+          <t>~-398.12 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~-0.83%</t>
+          <t>~-0.74%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14182,19 +14182,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>570.85</v>
+        <v>643.08</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~560.35 (unrealized)</t>
+          <t>~632.58 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~+1.09%</t>
+          <t>~+1.23%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14279,19 +14279,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>363.72</v>
+        <v>385.6</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~353.26 (unrealized)</t>
+          <t>~375.14 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~+0.70%</t>
+          <t>~+0.74%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14376,19 +14376,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>-37.57</v>
+        <v>-41.8</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~-47.75 (unrealized)</t>
+          <t>~-51.98 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~-1.11%</t>
+          <t>~-1.23%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
live pnl 2026-09-16 20:24 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -2323,17 +2323,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>#1ID LINK-USD SHORT</t>
+          <t>#1SW TRX-USD LONG</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>LINK-USD</t>
+          <t>TRX-USD</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2343,46 +2343,46 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>50.43</v>
+        <v>66.67</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>18.05</v>
+        <v>51.86</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>0</v>
+        <v>-27.64</v>
       </c>
       <c r="P27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>0</v>
+        <v>40.12</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>-67.76000000000001</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>0</v>
+        <v>-16.94</v>
       </c>
     </row>
     <row r="28">
@@ -2391,17 +2391,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>#1SW TRX-USD LONG</t>
+          <t>#1ID DOGE-USD SHORT</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>TRX-USD</t>
+          <t>DOGE-USD</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2411,46 +2411,46 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>66.67</v>
+        <v>50.67</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>51.86</v>
+        <v>31.42</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="N28" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>-27.64</v>
+        <v>-88.45</v>
       </c>
       <c r="P28" s="4" t="n">
-        <v>40.12</v>
+        <v>12.57</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>-67.76000000000001</v>
+        <v>-101.02</v>
       </c>
       <c r="R28" s="4" t="n">
-        <v>-16.94</v>
+        <v>-101.02</v>
       </c>
     </row>
     <row r="29">
@@ -2459,66 +2459,66 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>#1ID DOGE-USD SHORT</t>
+          <t>#5SW XLP LONG</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>DOGE-USD</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>Range&lt;1%+SMA20&lt;EMA20</t>
         </is>
       </c>
       <c r="H29" s="4" t="n">
-        <v>50.67</v>
+        <v>58.26</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>31.42</v>
+        <v>67.47</v>
       </c>
       <c r="J29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O29" s="4" t="n">
-        <v>-88.45</v>
+        <v>-149.74</v>
       </c>
       <c r="P29" s="4" t="n">
-        <v>12.57</v>
+        <v>20.27</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>-101.02</v>
+        <v>-170.01</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>-101.02</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="30">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>#5SW XLP LONG</t>
+          <t>#57SW XLRE LONG</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2552,41 +2552,41 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Range&lt;1%+SMA20&lt;EMA20</t>
+          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&lt;Open</t>
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>58.26</v>
+        <v>69.23</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>67.47</v>
+        <v>16.84</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O30" s="4" t="n">
-        <v>-149.74</v>
+        <v>-469.04</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>20.27</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>-170.01</v>
+        <v>-479</v>
       </c>
       <c r="R30" s="4" t="n">
-        <v>-85</v>
+        <v>-479</v>
       </c>
     </row>
     <row r="31">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>#57SW XLRE LONG</t>
+          <t>#3SW XLC LONG</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2620,20 +2620,20 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&lt;Open</t>
+          <t>Price&gt;EMA9+Range&lt;1%</t>
         </is>
       </c>
       <c r="H31" s="4" t="n">
-        <v>69.23</v>
+        <v>53.98</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>16.84</v>
+        <v>68.92</v>
       </c>
       <c r="J31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K31" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2645,16 +2645,16 @@
         <v>0</v>
       </c>
       <c r="O31" s="4" t="n">
-        <v>-469.04</v>
+        <v>-750.65</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>9.960000000000001</v>
+        <v>10.32</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>-479</v>
+        <v>-760.97</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>-479</v>
+        <v>-760.97</v>
       </c>
     </row>
     <row r="32">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>#3SW XLC LONG</t>
+          <t>#31SW QQQ LONG</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2688,20 +2688,20 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;EMA9+Range&lt;1%</t>
+          <t>Price&gt;SMA50+2Red</t>
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>53.98</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>68.92</v>
+        <v>48.57</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2713,16 +2713,16 @@
         <v>0</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-750.65</v>
+        <v>-865.8099999999999</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>10.32</v>
+        <v>10.46</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
       <c r="R32" s="4" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
     </row>
     <row r="33">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>#31SW QQQ LONG</t>
+          <t>#4SW OEF LONG</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>OEF</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2756,41 +2756,41 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+2Red</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
         </is>
       </c>
       <c r="H33" s="4" t="n">
-        <v>65.29000000000001</v>
+        <v>59.53</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>48.57</v>
+        <v>109.78</v>
       </c>
       <c r="J33" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K33" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="L33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="O33" s="4" t="n">
-        <v>-865.8099999999999</v>
+        <v>-982.38</v>
       </c>
       <c r="P33" s="4" t="n">
-        <v>10.46</v>
+        <v>50.18</v>
       </c>
       <c r="Q33" s="6" t="n">
-        <v>-876.27</v>
+        <v>-1032.56</v>
       </c>
       <c r="R33" s="4" t="n">
-        <v>-876.27</v>
+        <v>-206.51</v>
       </c>
     </row>
     <row r="34">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>#4SW OEF LONG</t>
+          <t>#5SW KBE LONG</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>OEF</t>
+          <t>KBE</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2824,41 +2824,41 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
+          <t>EMA9&lt;EMA50+Price&gt;EMA50</t>
         </is>
       </c>
       <c r="H34" s="4" t="n">
-        <v>59.53</v>
+        <v>50.67</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>109.78</v>
+        <v>17.55</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M34" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="N34" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O34" s="4" t="n">
-        <v>-982.38</v>
+        <v>-1039.2</v>
       </c>
       <c r="P34" s="4" t="n">
-        <v>50.18</v>
+        <v>10.29</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>-1032.56</v>
+        <v>-1049.49</v>
       </c>
       <c r="R34" s="4" t="n">
-        <v>-206.51</v>
+        <v>-1049.49</v>
       </c>
     </row>
     <row r="35">
@@ -2867,39 +2867,39 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>#5SW KBE LONG</t>
+          <t>#1ID LINK-USD SHORT</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>KBE</t>
+          <t>LINK-USD</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>EMA9&lt;EMA50+Price&gt;EMA50</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H35" s="4" t="n">
-        <v>50.67</v>
+        <v>50.43</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>17.55</v>
+        <v>18.05</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1</v>
@@ -2917,16 +2917,16 @@
         <v>0</v>
       </c>
       <c r="O35" s="4" t="n">
-        <v>-1039.2</v>
+        <v>-2489.46</v>
       </c>
       <c r="P35" s="4" t="n">
-        <v>10.29</v>
+        <v>360.6</v>
       </c>
       <c r="Q35" s="6" t="n">
-        <v>-1049.49</v>
+        <v>-2850.06</v>
       </c>
       <c r="R35" s="4" t="n">
-        <v>-1049.49</v>
+        <v>-2850.06</v>
       </c>
     </row>
     <row r="36">
@@ -14082,27 +14082,29 @@
           <t>12</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="L2" s="2" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:54:37 IST</t>
+        </is>
+      </c>
       <c r="N2" s="4" t="n">
-        <v>-1150.61</v>
+        <v>-2489.46</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>360.6</v>
       </c>
-      <c r="P2" s="9" t="inlineStr">
-        <is>
-          <t>~-1,511.21 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q2" s="9" t="inlineStr">
-        <is>
-          <t>~-0.96%</t>
-        </is>
+      <c r="P2" s="6" t="n">
+        <v>-2850.06</v>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>-2.37</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -14127,7 +14129,7 @@
       </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
-          <t>#1ID Price&gt;SMA20+RSI&lt;45</t>
+          <t>#1ID Price&gt;SMA20+RSI&lt;45 | 🎯 SL Hit (live)</t>
         </is>
       </c>
     </row>
@@ -20745,18 +20747,18 @@
       <c r="L70" s="15" t="inlineStr"/>
       <c r="M70" s="14" t="inlineStr"/>
       <c r="N70" s="17" t="n">
-        <v>25910.85</v>
+        <v>23421.39</v>
       </c>
       <c r="O70" s="17" t="n">
-        <v>2459.59</v>
+        <v>2820.19</v>
       </c>
       <c r="P70" s="18" t="n">
-        <v>23451.26</v>
+        <v>20601.2</v>
       </c>
       <c r="Q70" s="16" t="inlineStr"/>
       <c r="R70" s="15" t="inlineStr">
         <is>
-          <t>68 trades (62 closed / 6 open)</t>
+          <t>68 trades (63 closed / 5 open)</t>
         </is>
       </c>
       <c r="S70" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 21:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14184,19 +14184,19 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="4" t="n">
-        <v>-105.08</v>
+        <v>56.8</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>~-115.52 (unrealized)</t>
+          <t>~46.36 (unrealized)</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>~-0.20%</t>
+          <t>~+0.11%</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -14281,19 +14281,19 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="4" t="n">
-        <v>-912.42</v>
+        <v>-761.72</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>~-922.84 (unrealized)</t>
+          <t>~-772.14 (unrealized)</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>~-1.75%</t>
+          <t>~-1.46%</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -14378,19 +14378,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>33.55</v>
+        <v>181.74</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~23.05 (unrealized)</t>
+          <t>~171.24 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+0.06%</t>
+          <t>~+0.35%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14475,19 +14475,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-18.81</v>
+        <v>-37.62</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~-29.27 (unrealized)</t>
+          <t>~-48.08 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>~-0.04%</t>
+          <t>~-0.07%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14572,19 +14572,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-41.56</v>
+        <v>-35.1</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-51.74 (unrealized)</t>
+          <t>~-45.28 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-1.22%</t>
+          <t>~-1.03%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-16 22:14 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14572,19 +14572,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-35.1</v>
+        <v>-36.77</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-45.28 (unrealized)</t>
+          <t>~-46.95 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-1.03%</t>
+          <t>~-1.08%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
live pnl 2026-09-16 23:41 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -2323,17 +2323,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>#1ID XRP-USD SHORT</t>
+          <t>#1SW TRX-USD LONG</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>XRP-USD</t>
+          <t>TRX-USD</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2343,46 +2343,46 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>48.15</v>
+        <v>66.67</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>5.91</v>
+        <v>51.86</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>0</v>
+        <v>-27.64</v>
       </c>
       <c r="P27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>0</v>
+        <v>40.12</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>-67.76000000000001</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>0</v>
+        <v>-16.94</v>
       </c>
     </row>
     <row r="28">
@@ -2391,17 +2391,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>#1SW TRX-USD LONG</t>
+          <t>#1ID DOGE-USD SHORT</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>TRX-USD</t>
+          <t>DOGE-USD</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2411,46 +2411,46 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>66.67</v>
+        <v>50.67</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>51.86</v>
+        <v>31.42</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="N28" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>-27.64</v>
+        <v>-88.45</v>
       </c>
       <c r="P28" s="4" t="n">
-        <v>40.12</v>
+        <v>12.57</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>-67.76000000000001</v>
+        <v>-101.02</v>
       </c>
       <c r="R28" s="4" t="n">
-        <v>-16.94</v>
+        <v>-101.02</v>
       </c>
     </row>
     <row r="29">
@@ -2459,66 +2459,66 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>#1ID DOGE-USD SHORT</t>
+          <t>#5SW XLP LONG</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>DOGE-USD</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>Range&lt;1%+SMA20&lt;EMA20</t>
         </is>
       </c>
       <c r="H29" s="4" t="n">
-        <v>50.67</v>
+        <v>58.26</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>31.42</v>
+        <v>67.47</v>
       </c>
       <c r="J29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O29" s="4" t="n">
-        <v>-88.45</v>
+        <v>-149.74</v>
       </c>
       <c r="P29" s="4" t="n">
-        <v>12.57</v>
+        <v>20.27</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>-101.02</v>
+        <v>-170.01</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>-101.02</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="30">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>#5SW XLP LONG</t>
+          <t>#57SW XLRE LONG</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2552,41 +2552,41 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Range&lt;1%+SMA20&lt;EMA20</t>
+          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&lt;Open</t>
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>58.26</v>
+        <v>69.23</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>67.47</v>
+        <v>16.84</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O30" s="4" t="n">
-        <v>-149.74</v>
+        <v>-469.04</v>
       </c>
       <c r="P30" s="4" t="n">
-        <v>20.27</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>-170.01</v>
+        <v>-479</v>
       </c>
       <c r="R30" s="4" t="n">
-        <v>-85</v>
+        <v>-479</v>
       </c>
     </row>
     <row r="31">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>#57SW XLRE LONG</t>
+          <t>#3SW XLC LONG</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2620,20 +2620,20 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&lt;Open</t>
+          <t>Price&gt;EMA9+Range&lt;1%</t>
         </is>
       </c>
       <c r="H31" s="4" t="n">
-        <v>69.23</v>
+        <v>53.98</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>16.84</v>
+        <v>68.92</v>
       </c>
       <c r="J31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="K31" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2645,16 +2645,16 @@
         <v>0</v>
       </c>
       <c r="O31" s="4" t="n">
-        <v>-469.04</v>
+        <v>-750.65</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>9.960000000000001</v>
+        <v>10.32</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>-479</v>
+        <v>-760.97</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>-479</v>
+        <v>-760.97</v>
       </c>
     </row>
     <row r="32">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>#3SW XLC LONG</t>
+          <t>#31SW QQQ LONG</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2688,20 +2688,20 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;EMA9+Range&lt;1%</t>
+          <t>Price&gt;SMA50+2Red</t>
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>53.98</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>68.92</v>
+        <v>48.57</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2713,16 +2713,16 @@
         <v>0</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-750.65</v>
+        <v>-865.8099999999999</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>10.32</v>
+        <v>10.46</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
       <c r="R32" s="4" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
     </row>
     <row r="33">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>#31SW QQQ LONG</t>
+          <t>#4SW OEF LONG</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>OEF</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2756,41 +2756,41 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+2Red</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
         </is>
       </c>
       <c r="H33" s="4" t="n">
-        <v>65.29000000000001</v>
+        <v>59.53</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>48.57</v>
+        <v>109.78</v>
       </c>
       <c r="J33" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K33" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="L33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="O33" s="4" t="n">
-        <v>-865.8099999999999</v>
+        <v>-982.38</v>
       </c>
       <c r="P33" s="4" t="n">
-        <v>10.46</v>
+        <v>50.18</v>
       </c>
       <c r="Q33" s="6" t="n">
-        <v>-876.27</v>
+        <v>-1032.56</v>
       </c>
       <c r="R33" s="4" t="n">
-        <v>-876.27</v>
+        <v>-206.51</v>
       </c>
     </row>
     <row r="34">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>#4SW OEF LONG</t>
+          <t>#5SW KBE LONG</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>OEF</t>
+          <t>KBE</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2824,41 +2824,41 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
+          <t>EMA9&lt;EMA50+Price&gt;EMA50</t>
         </is>
       </c>
       <c r="H34" s="4" t="n">
-        <v>59.53</v>
+        <v>50.67</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>109.78</v>
+        <v>17.55</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M34" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="N34" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="O34" s="4" t="n">
-        <v>-982.38</v>
+        <v>-1039.2</v>
       </c>
       <c r="P34" s="4" t="n">
-        <v>50.18</v>
+        <v>10.29</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>-1032.56</v>
+        <v>-1049.49</v>
       </c>
       <c r="R34" s="4" t="n">
-        <v>-206.51</v>
+        <v>-1049.49</v>
       </c>
     </row>
     <row r="35">
@@ -2867,39 +2867,39 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>#5SW KBE LONG</t>
+          <t>#1ID LINK-USD SHORT</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>KBE</t>
+          <t>LINK-USD</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>EMA9&lt;EMA50+Price&gt;EMA50</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H35" s="4" t="n">
-        <v>50.67</v>
+        <v>50.43</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>17.55</v>
+        <v>18.05</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1</v>
@@ -2917,16 +2917,16 @@
         <v>0</v>
       </c>
       <c r="O35" s="4" t="n">
-        <v>-1039.2</v>
+        <v>-2489.46</v>
       </c>
       <c r="P35" s="4" t="n">
-        <v>10.29</v>
+        <v>360.6</v>
       </c>
       <c r="Q35" s="6" t="n">
-        <v>-1049.49</v>
+        <v>-2850.06</v>
       </c>
       <c r="R35" s="4" t="n">
-        <v>-1049.49</v>
+        <v>-2850.06</v>
       </c>
     </row>
     <row r="36">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>#1ID LINK-USD SHORT</t>
+          <t>#1ID XRP-USD SHORT</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>LINK-USD</t>
+          <t>XRP-USD</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2964,10 +2964,10 @@
         </is>
       </c>
       <c r="H36" s="4" t="n">
-        <v>50.43</v>
+        <v>48.15</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>18.05</v>
+        <v>5.91</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>1</v>
@@ -2985,16 +2985,16 @@
         <v>0</v>
       </c>
       <c r="O36" s="4" t="n">
-        <v>-2489.46</v>
+        <v>-2502.38</v>
       </c>
       <c r="P36" s="4" t="n">
-        <v>360.6</v>
+        <v>402.06</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>-2850.06</v>
+        <v>-2904.44</v>
       </c>
       <c r="R36" s="4" t="n">
-        <v>-2850.06</v>
+        <v>-2904.44</v>
       </c>
     </row>
     <row r="37">
@@ -14082,27 +14082,29 @@
           <t>12</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="L2" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17 05:11:30 IST</t>
+        </is>
+      </c>
       <c r="N2" s="4" t="n">
-        <v>-649.16</v>
+        <v>-2502.38</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>402.06</v>
       </c>
-      <c r="P2" s="9" t="inlineStr">
-        <is>
-          <t>~-1,051.22 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q2" s="9" t="inlineStr">
-        <is>
-          <t>~-0.48%</t>
-        </is>
+      <c r="P2" s="6" t="n">
+        <v>-2904.44</v>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>-2.17</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -14127,7 +14129,7 @@
       </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
-          <t>#1ID Price&gt;SMA20+RSI&lt;45</t>
+          <t>#1ID Price&gt;SMA20+RSI&lt;45 | 🎯 SL Hit (live)</t>
         </is>
       </c>
     </row>
@@ -20941,18 +20943,18 @@
       <c r="L72" s="15" t="inlineStr"/>
       <c r="M72" s="14" t="inlineStr"/>
       <c r="N72" s="17" t="n">
-        <v>23421.39</v>
+        <v>20919.01</v>
       </c>
       <c r="O72" s="17" t="n">
-        <v>2820.19</v>
+        <v>3222.25</v>
       </c>
       <c r="P72" s="18" t="n">
-        <v>20601.2</v>
+        <v>17696.76</v>
       </c>
       <c r="Q72" s="16" t="inlineStr"/>
       <c r="R72" s="15" t="inlineStr">
         <is>
-          <t>70 trades (63 closed / 7 open)</t>
+          <t>70 trades (64 closed / 6 open)</t>
         </is>
       </c>
       <c r="S72" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
live pnl 2026-09-17 00:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -759,45 +759,45 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>#1ID SOL-USD SHORT</t>
+          <t>#3SW XLE LONG</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>SOL-USD</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA20+RSI&lt;50</t>
+          <t>EMA9&gt;EMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
-        <v>47.24</v>
+        <v>51.28</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>23.69</v>
+        <v>18.74</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>2</v>
@@ -809,16 +809,16 @@
         <v>100</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3782.21</v>
+        <v>2085.52</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>573.08</v>
+        <v>20.2</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>3209.13</v>
+        <v>2065.32</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>1604.57</v>
+        <v>1032.66</v>
       </c>
     </row>
     <row r="5">
@@ -827,7 +827,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>#3SW XLE LONG</t>
+          <t>#52SW QQQ LONG</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -852,23 +852,23 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA50+Range&lt;1%</t>
+          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&gt;Open</t>
         </is>
       </c>
       <c r="H5" s="4" t="n">
-        <v>51.28</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>18.74</v>
+        <v>18.68</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -877,16 +877,16 @@
         <v>100</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>2085.52</v>
+        <v>1989.42</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>20.2</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>2065.32</v>
+        <v>1979.47</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>1032.66</v>
+        <v>1979.47</v>
       </c>
     </row>
     <row r="6">
@@ -895,12 +895,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>#52SW QQQ LONG</t>
+          <t>#5ID QQQ LONG</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -920,23 +920,23 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+EMA9&lt;EMA20+Close&gt;Open</t>
+          <t>Price&gt;SMA20+Price&lt;SMA50+EMA9&gt;EMA20+EMA20&lt;EMA50</t>
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>71.43000000000001</v>
+        <v>63.38</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>18.68</v>
+        <v>11.65</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>0</v>
@@ -945,16 +945,16 @@
         <v>100</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>1989.42</v>
+        <v>1610.54</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>9.949999999999999</v>
+        <v>36.37</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>1979.47</v>
+        <v>1574.17</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>1979.47</v>
+        <v>787.09</v>
       </c>
     </row>
     <row r="7">
@@ -963,17 +963,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>#5ID QQQ LONG</t>
+          <t>#28SW XLK LONG</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -988,20 +988,20 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+Price&lt;SMA50+EMA9&gt;EMA20+EMA20&lt;EMA50</t>
+          <t>Price&gt;SMA50+EMA20&gt;EMA50+2Red</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>63.38</v>
+        <v>63.73</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>11.65</v>
+        <v>50.46</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>2</v>
@@ -1013,16 +1013,16 @@
         <v>100</v>
       </c>
       <c r="O7" s="4" t="n">
-        <v>1610.54</v>
+        <v>1450.08</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>36.37</v>
+        <v>20.1</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>1574.17</v>
+        <v>1429.98</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>787.09</v>
+        <v>714.99</v>
       </c>
     </row>
     <row r="8">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>#28SW XLK LONG</t>
+          <t>#4SW XLV LONG</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1056,41 +1056,41 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+EMA20&gt;EMA50+2Red</t>
+          <t>EMA9&gt;EMA20+Range&lt;1%</t>
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>63.73</v>
+        <v>52.32</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>50.46</v>
+        <v>23.85</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M8" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="N8" s="2" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1450.08</v>
+        <v>1420.63</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>20.1</v>
+        <v>61.23</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>1429.98</v>
+        <v>1359.4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>714.99</v>
+        <v>226.57</v>
       </c>
     </row>
     <row r="9">
@@ -1099,17 +1099,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>#4SW XLV LONG</t>
+          <t>#14ID IWM SHORT</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1119,46 +1119,46 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Range&lt;1%</t>
+          <t>Price&lt;SMA50+EMA9&gt;EMA20+EMA20&lt;EMA50+Close&gt;Open</t>
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>52.32</v>
+        <v>63.41</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>23.85</v>
+        <v>7.5</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="O9" s="4" t="n">
-        <v>1420.63</v>
+        <v>1182.87</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>61.23</v>
+        <v>19.75</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>1359.4</v>
+        <v>1163.12</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>226.57</v>
+        <v>1163.12</v>
       </c>
     </row>
     <row r="10">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>#14ID IWM SHORT</t>
+          <t>#36ID DIA LONG</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1187,46 +1187,46 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Price&lt;SMA50+EMA9&gt;EMA20+EMA20&lt;EMA50+Close&gt;Open</t>
+          <t>Price&lt;SMA50+EMA9&gt;EMA20+Close&lt;Open+2Red</t>
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>63.41</v>
+        <v>67.86</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>7.5</v>
+        <v>2.52</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1182.87</v>
+        <v>1221.22</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>19.75</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>1163.12</v>
+        <v>1144.54</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1163.12</v>
+        <v>286.13</v>
       </c>
     </row>
     <row r="11">
@@ -1235,22 +1235,22 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>#36ID DIA LONG</t>
+          <t>#935LB NSE LONG</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>LONG_BOUNCE_5m</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>NSE</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>INDIAN</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1260,41 +1260,41 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Price&lt;SMA50+EMA9&gt;EMA20+Close&lt;Open+2Red</t>
+          <t>Long L1: 5m -3.5%/90m vol2.5x RSI&lt;=45 gap1.5 below-VWAP&amp;down 10:30-12:30</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>67.86</v>
+        <v>54.3</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>2.52</v>
+        <v>56</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>50</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>1221.22</v>
+        <v>1223.5</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>76.68000000000001</v>
+        <v>377.69</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>1144.54</v>
+        <v>845.8099999999999</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>286.13</v>
+        <v>422.9</v>
       </c>
     </row>
     <row r="12">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>#935LB NSE LONG</t>
+          <t>#31ID SPY LONG</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>LONG_BOUNCE_5m</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>NSE</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>INDIAN</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1328,17 +1328,17 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Long L1: 5m -3.5%/90m vol2.5x RSI&lt;=45 gap1.5 below-VWAP&amp;down 10:30-12:30</t>
+          <t>Price&gt;SMA50+EMA20&lt;EMA50+Close&lt;Open</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>54.3</v>
+        <v>63.16</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>56</v>
+        <v>3.67</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1347,22 +1347,22 @@
         <v>1</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1223.5</v>
+        <v>696.96</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>377.69</v>
+        <v>17.95</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>845.8099999999999</v>
+        <v>679.01</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>422.9</v>
+        <v>679.01</v>
       </c>
     </row>
     <row r="13">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>#31ID SPY LONG</t>
+          <t>#1SW XLY LONG</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1396,14 +1396,14 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+EMA20&lt;EMA50+Close&lt;Open</t>
+          <t>EMA9&lt;EMA50+RSI&gt;50</t>
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>63.16</v>
+        <v>58.65</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>3.67</v>
+        <v>59.99</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1</v>
@@ -1421,16 +1421,16 @@
         <v>100</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>696.96</v>
+        <v>633.37</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>17.95</v>
+        <v>9.94</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>679.01</v>
+        <v>623.4299999999999</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>679.01</v>
+        <v>623.4299999999999</v>
       </c>
     </row>
     <row r="14">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>#1SW XLY LONG</t>
+          <t>#37SW QQQ LONG</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1464,17 +1464,17 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>EMA9&lt;EMA50+RSI&gt;50</t>
+          <t>Price&gt;SMA50+EMA9&gt;EMA20+2Red</t>
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>58.65</v>
+        <v>60.94</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>59.99</v>
+        <v>45.8</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1483,22 +1483,22 @@
         <v>1</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>633.37</v>
+        <v>633.8</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>9.94</v>
+        <v>19.8</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>623.4299999999999</v>
+        <v>614</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>623.4299999999999</v>
+        <v>307</v>
       </c>
     </row>
     <row r="15">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>#37SW QQQ LONG</t>
+          <t>#14SW ETH-USD LONG</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1517,12 +1517,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ETH-USD</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1532,14 +1532,14 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+EMA9&gt;EMA20+2Red</t>
+          <t>Price&gt;SMA50+Range&gt;1.5%+2Red</t>
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>60.94</v>
+        <v>63.36</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>45.8</v>
+        <v>74.7</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>2</v>
@@ -1557,16 +1557,16 @@
         <v>50</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>633.8</v>
+        <v>777.78</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>19.8</v>
+        <v>285.41</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>614</v>
+        <v>492.37</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>307</v>
+        <v>246.18</v>
       </c>
     </row>
     <row r="16">
@@ -1575,17 +1575,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>#14SW ETH-USD LONG</t>
+          <t>#1ID SOL-USD SHORT</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>ETH-USD</t>
+          <t>SOL-USD</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1595,46 +1595,46 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+Range&gt;1.5%+2Red</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA20+RSI&lt;50</t>
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>63.36</v>
+        <v>47.24</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>74.7</v>
+        <v>23.69</v>
       </c>
       <c r="J16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>777.78</v>
+        <v>1386.59</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>285.41</v>
+        <v>943.16</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>492.37</v>
+        <v>443.43</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>246.18</v>
+        <v>147.81</v>
       </c>
     </row>
     <row r="17">
@@ -14181,27 +14181,29 @@
           <t>12</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="L3" s="2" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17 05:42:32 IST</t>
+        </is>
+      </c>
       <c r="N3" s="4" t="n">
-        <v>-571.05</v>
+        <v>-2395.62</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>370.08</v>
       </c>
-      <c r="P3" s="9" t="inlineStr">
-        <is>
-          <t>~-941.13 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>~-0.46%</t>
-        </is>
+      <c r="P3" s="6" t="n">
+        <v>-2765.7</v>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>-2.24</v>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -14226,7 +14228,7 @@
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
-          <t>#1ID EMA9&gt;EMA20+Price&gt;SMA20+RSI&lt;50</t>
+          <t>#1ID EMA9&gt;EMA20+Price&gt;SMA20+RSI&lt;50 | 🎯 SL Hit (live)</t>
         </is>
       </c>
     </row>
@@ -20943,18 +20945,18 @@
       <c r="L72" s="15" t="inlineStr"/>
       <c r="M72" s="14" t="inlineStr"/>
       <c r="N72" s="17" t="n">
-        <v>20919.01</v>
+        <v>18523.39</v>
       </c>
       <c r="O72" s="17" t="n">
-        <v>3222.25</v>
+        <v>3592.33</v>
       </c>
       <c r="P72" s="18" t="n">
-        <v>17696.76</v>
+        <v>14931.06</v>
       </c>
       <c r="Q72" s="16" t="inlineStr"/>
       <c r="R72" s="15" t="inlineStr">
         <is>
-          <t>70 trades (64 closed / 6 open)</t>
+          <t>70 trades (65 closed / 5 open)</t>
         </is>
       </c>
       <c r="S72" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 05:08 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-42.44</v>
+        <v>-38.34</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-52.62 (unrealized)</t>
+          <t>~-48.52 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.25%</t>
+          <t>~-1.13%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 05:57 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-38.34</v>
+        <v>-40.73</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-48.52 (unrealized)</t>
+          <t>~-50.91 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.13%</t>
+          <t>~-1.20%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 09:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-40.73</v>
+        <v>-44.05</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-50.91 (unrealized)</t>
+          <t>~-54.23 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.20%</t>
+          <t>~-1.30%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 14:58 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14382,19 +14382,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>56.8</v>
+        <v>1174.34</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~46.36 (unrealized)</t>
+          <t>~1,163.90 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+0.11%</t>
+          <t>~+2.25%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-761.72</v>
+        <v>-253.45</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~-772.14 (unrealized)</t>
+          <t>~-263.87 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>~-1.46%</t>
+          <t>~-0.49%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>181.74</v>
+        <v>-65.23999999999999</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~171.24 (unrealized)</t>
+          <t>~-75.74 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~+0.35%</t>
+          <t>~-0.12%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14673,19 +14673,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>-37.62</v>
+        <v>-231.99</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>~-48.08 (unrealized)</t>
+          <t>~-242.45 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>~-0.07%</t>
+          <t>~-0.44%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-44.05</v>
+        <v>-50.17</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-54.23 (unrealized)</t>
+          <t>~-60.35 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.30%</t>
+          <t>~-1.48%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 17:12 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14382,19 +14382,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>1174.34</v>
+        <v>1232.56</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~1,163.90 (unrealized)</t>
+          <t>~1,222.12 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+2.25%</t>
+          <t>~+2.36%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-253.45</v>
+        <v>-149.33</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~-263.87 (unrealized)</t>
+          <t>~-159.75 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>~-0.49%</t>
+          <t>~-0.29%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-65.23999999999999</v>
+        <v>-93.2</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-75.74 (unrealized)</t>
+          <t>~-103.70 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-0.12%</t>
+          <t>~-0.18%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14673,19 +14673,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>-231.99</v>
+        <v>-25.08</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>~-242.45 (unrealized)</t>
+          <t>~-35.54 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>~-0.44%</t>
+          <t>~-0.05%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-50.17</v>
+        <v>-55.02</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-60.35 (unrealized)</t>
+          <t>~-65.20 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.48%</t>
+          <t>~-1.62%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 17:42 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14382,19 +14382,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>1232.56</v>
+        <v>1215.52</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~1,222.12 (unrealized)</t>
+          <t>~1,205.08 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+2.36%</t>
+          <t>~+2.33%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14479,14 +14479,14 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-149.33</v>
+        <v>-152.07</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~-159.75 (unrealized)</t>
+          <t>~-162.49 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-93.2</v>
+        <v>-74.56</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-103.70 (unrealized)</t>
+          <t>~-85.06 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-0.18%</t>
+          <t>~-0.14%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14673,19 +14673,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>-25.08</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>~-35.54 (unrealized)</t>
+          <t>~61.64 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>~-0.05%</t>
+          <t>~+0.14%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-55.02</v>
+        <v>-55.66</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-65.20 (unrealized)</t>
+          <t>~-65.84 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.62%</t>
+          <t>~-1.64%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 18:28 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14382,19 +14382,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>1215.52</v>
+        <v>1209.84</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~1,205.08 (unrealized)</t>
+          <t>~1,199.40 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+2.33%</t>
+          <t>~+2.32%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-152.07</v>
+        <v>-126.04</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~-162.49 (unrealized)</t>
+          <t>~-136.46 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>~-0.29%</t>
+          <t>~-0.24%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-74.56</v>
+        <v>-83.88</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-85.06 (unrealized)</t>
+          <t>~-94.38 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-0.14%</t>
+          <t>~-0.16%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14673,19 +14673,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>72.09999999999999</v>
+        <v>59.57</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>~61.64 (unrealized)</t>
+          <t>~49.11 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>~+0.14%</t>
+          <t>~+0.11%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-55.66</v>
+        <v>-58.09</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-65.84 (unrealized)</t>
+          <t>~-68.27 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~-1.64%</t>
+          <t>~-1.71%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 19:08 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14382,19 +14382,19 @@
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="4" t="n">
-        <v>1209.84</v>
+        <v>1275.16</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>~1,199.40 (unrealized)</t>
+          <t>~1,264.72 (unrealized)</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>~+2.32%</t>
+          <t>~+2.44%</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>-126.04</v>
+        <v>-100.01</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~-136.46 (unrealized)</t>
+          <t>~-110.43 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>~-0.24%</t>
+          <t>~-0.19%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-83.88</v>
+        <v>-149.12</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-94.38 (unrealized)</t>
+          <t>~-159.62 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-0.16%</t>
+          <t>~-0.28%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14673,19 +14673,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>59.57</v>
+        <v>81.51000000000001</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>~49.11 (unrealized)</t>
+          <t>~71.05 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>~+0.11%</t>
+          <t>~+0.16%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14770,14 +14770,14 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>-58.09</v>
+        <v>-57.97</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~-68.27 (unrealized)</t>
+          <t>~-68.15 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 21:14 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14085,19 +14085,19 @@
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="4" t="n">
-        <v>26.1</v>
+        <v>-20.88</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>39.82</v>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>~-13.72 (unrealized)</t>
+          <t>~-60.70 (unrealized)</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>~+0.01%</t>
+          <t>~-0.01%</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -14479,19 +14479,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>1255.28</v>
+        <v>1221.2</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>~1,244.84 (unrealized)</t>
+          <t>~1,210.76 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>~+2.41%</t>
+          <t>~+2.34%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14576,19 +14576,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-94.53</v>
+        <v>-101.38</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>~-104.95 (unrealized)</t>
+          <t>~-111.80 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>~-0.18%</t>
+          <t>~-0.19%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14673,19 +14673,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>-116.5</v>
+        <v>-121.16</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>~-127.00 (unrealized)</t>
+          <t>~-131.66 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>~-0.22%</t>
+          <t>~-0.23%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14770,19 +14770,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>40.76</v>
+        <v>62.7</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>~30.30 (unrealized)</t>
+          <t>~52.24 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>~+0.08%</t>
+          <t>~+0.12%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-46.6</v>
+        <v>-43.87</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~-56.78 (unrealized)</t>
+          <t>~-54.05 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~-1.37%</t>
+          <t>~-1.29%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 22:17 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-43.87</v>
+        <v>-49.29</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~-54.05 (unrealized)</t>
+          <t>~-59.47 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~-1.29%</t>
+          <t>~-1.45%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-17 23:00 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-49.29</v>
+        <v>-47.4</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~-59.47 (unrealized)</t>
+          <t>~-57.58 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~-1.45%</t>
+          <t>~-1.40%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-18 05:33 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-47.4</v>
+        <v>-35.57</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~-57.58 (unrealized)</t>
+          <t>~-45.75 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~-1.40%</t>
+          <t>~-1.05%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-18 05:44 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-35.57</v>
+        <v>-35.21</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~-45.75 (unrealized)</t>
+          <t>~-45.39 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~-1.05%</t>
+          <t>~-1.04%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-18 08:45 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14867,19 +14867,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-35.21</v>
+        <v>-27.81</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>~-45.39 (unrealized)</t>
+          <t>~-37.99 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>~-1.04%</t>
+          <t>~-0.82%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
live pnl 2026-09-18 19:17 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -109,6 +109,9 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -119,9 +122,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1303,17 +1303,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>#31ID SPY LONG</t>
+          <t>#1SW XLY LONG</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1328,20 +1328,20 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+EMA20&lt;EMA50+Close&lt;Open</t>
+          <t>EMA9&lt;EMA50+RSI&gt;50</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>63.16</v>
+        <v>58.65</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>3.67</v>
+        <v>59.99</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>1</v>
@@ -1353,16 +1353,16 @@
         <v>100</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>696.96</v>
+        <v>633.37</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>17.95</v>
+        <v>9.94</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>679.01</v>
+        <v>623.4299999999999</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>679.01</v>
+        <v>623.4299999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>#1SW XLY LONG</t>
+          <t>#37SW QQQ LONG</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1396,17 +1396,17 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>EMA9&lt;EMA50+RSI&gt;50</t>
+          <t>Price&gt;SMA50+EMA9&gt;EMA20+2Red</t>
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>58.65</v>
+        <v>60.94</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>59.99</v>
+        <v>45.8</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1415,22 +1415,22 @@
         <v>1</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O13" s="4" t="n">
-        <v>633.37</v>
+        <v>633.8</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>9.94</v>
+        <v>19.8</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>623.4299999999999</v>
+        <v>614</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>623.4299999999999</v>
+        <v>307</v>
       </c>
     </row>
     <row r="14">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>#37SW QQQ LONG</t>
+          <t>#14SW ETH-USD LONG</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1449,12 +1449,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>ETH-USD</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1464,14 +1464,14 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+EMA9&gt;EMA20+2Red</t>
+          <t>Price&gt;SMA50+Range&gt;1.5%+2Red</t>
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>60.94</v>
+        <v>63.36</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>45.8</v>
+        <v>74.7</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>2</v>
@@ -1489,16 +1489,16 @@
         <v>50</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>633.8</v>
+        <v>777.78</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>19.8</v>
+        <v>285.41</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>614</v>
+        <v>492.37</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>307</v>
+        <v>246.18</v>
       </c>
     </row>
     <row r="15">
@@ -1507,17 +1507,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>#14SW ETH-USD LONG</t>
+          <t>#1ID SOL-USD SHORT</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>ETH-USD</t>
+          <t>SOL-USD</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1527,46 +1527,46 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+Range&gt;1.5%+2Red</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA20+RSI&lt;50</t>
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>63.36</v>
+        <v>47.24</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>74.7</v>
+        <v>23.69</v>
       </c>
       <c r="J15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="K15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="M15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>777.78</v>
+        <v>1386.59</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>285.41</v>
+        <v>943.16</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>492.37</v>
+        <v>443.43</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>246.18</v>
+        <v>147.81</v>
       </c>
     </row>
     <row r="16">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>#1ID SOL-USD SHORT</t>
+          <t>#32ID SPY LONG</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1585,56 +1585,56 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>SOL-USD</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA20+RSI&lt;50</t>
+          <t>Price&gt;SMA20+EMA9&gt;EMA20+EMA20&lt;EMA50+Close&gt;Open</t>
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>47.24</v>
+        <v>60.24</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>23.69</v>
+        <v>3.27</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>1386.59</v>
+        <v>410.34</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>943.16</v>
+        <v>37.47</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>443.43</v>
+        <v>372.87</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>147.81</v>
+        <v>186.43</v>
       </c>
     </row>
     <row r="17">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>#32ID SPY LONG</t>
+          <t>#16ID SPY LONG</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1672,13 +1672,13 @@
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>60.24</v>
+        <v>62.35</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>3.27</v>
+        <v>6.99</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -1687,22 +1687,22 @@
         <v>1</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>410.34</v>
+        <v>373.46</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>37.47</v>
+        <v>20.86</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>372.87</v>
+        <v>352.6</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>186.43</v>
+        <v>352.6</v>
       </c>
     </row>
     <row r="18">
@@ -1711,17 +1711,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>#16ID SPY LONG</t>
+          <t>#5SW XLB LONG</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1736,14 +1736,14 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+EMA9&gt;EMA20+EMA20&lt;EMA50+Close&gt;Open</t>
+          <t>EMA9&gt;EMA20+Range&lt;1%</t>
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>62.35</v>
+        <v>50.21</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>6.99</v>
+        <v>11.26</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1</v>
@@ -1761,16 +1761,16 @@
         <v>100</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>373.46</v>
+        <v>342.69</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>20.86</v>
+        <v>10.06</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>352.6</v>
+        <v>332.63</v>
       </c>
       <c r="R18" s="4" t="n">
-        <v>352.6</v>
+        <v>332.63</v>
       </c>
     </row>
     <row r="19">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>#5SW XLB LONG</t>
+          <t>#2SW XLB LONG</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1804,17 +1804,17 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Range&lt;1%</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
         </is>
       </c>
       <c r="H19" s="4" t="n">
-        <v>50.21</v>
+        <v>51.71</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>11.26</v>
+        <v>23.19</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1823,22 +1823,22 @@
         <v>1</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>342.69</v>
+        <v>318.81</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>10.06</v>
+        <v>20.44</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>332.63</v>
+        <v>298.37</v>
       </c>
       <c r="R19" s="4" t="n">
-        <v>332.63</v>
+        <v>149.19</v>
       </c>
     </row>
     <row r="20">
@@ -1847,17 +1847,17 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>#2SW XLB LONG</t>
+          <t>#13ID DIA LONG</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1872,17 +1872,17 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
+          <t>RSI&lt;45+EMA20&gt;EMA50+Close&lt;Open+2Red</t>
         </is>
       </c>
       <c r="H20" s="4" t="n">
-        <v>51.71</v>
+        <v>60.16</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>23.19</v>
+        <v>7.88</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
@@ -1891,22 +1891,22 @@
         <v>1</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>318.81</v>
+        <v>316.83</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>20.44</v>
+        <v>18.54</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>298.37</v>
+        <v>298.29</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>149.19</v>
+        <v>298.29</v>
       </c>
     </row>
     <row r="21">
@@ -1915,17 +1915,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>#13ID DIA LONG</t>
+          <t>#3SW VTI LONG</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>VTI</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1940,14 +1940,14 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>RSI&lt;45+EMA20&gt;EMA50+Close&lt;Open+2Red</t>
+          <t>Range&lt;1%+SMA20&lt;EMA20</t>
         </is>
       </c>
       <c r="H21" s="4" t="n">
-        <v>60.16</v>
+        <v>60.9</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>7.88</v>
+        <v>112.53</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1</v>
@@ -1965,16 +1965,16 @@
         <v>100</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>316.83</v>
+        <v>294.2</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>18.54</v>
+        <v>10.03</v>
       </c>
       <c r="Q21" s="5" t="n">
-        <v>298.29</v>
+        <v>284.17</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>298.29</v>
+        <v>284.17</v>
       </c>
     </row>
     <row r="22">
@@ -1983,17 +1983,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>#3SW VTI LONG</t>
+          <t>#31ID SPY LONG</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>VTI</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2008,17 +2008,17 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Range&lt;1%+SMA20&lt;EMA20</t>
+          <t>Price&gt;SMA50+EMA20&lt;EMA50+Close&lt;Open</t>
         </is>
       </c>
       <c r="H22" s="4" t="n">
-        <v>60.9</v>
+        <v>63.16</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>112.53</v>
+        <v>3.67</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -2027,22 +2027,22 @@
         <v>1</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>294.2</v>
+        <v>244.84</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>10.03</v>
+        <v>57.77</v>
       </c>
       <c r="Q22" s="5" t="n">
-        <v>284.17</v>
+        <v>187.07</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>284.17</v>
+        <v>93.53</v>
       </c>
     </row>
     <row r="23">
@@ -14082,27 +14082,29 @@
           <t>6</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="L2" s="2" t="n">
+        <v>761.03</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19 00:47:46 IST</t>
+        </is>
+      </c>
       <c r="N2" s="4" t="n">
-        <v>-20.88</v>
+        <v>-452.12</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>39.82</v>
       </c>
-      <c r="P2" s="9" t="inlineStr">
-        <is>
-          <t>~-60.70 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q2" s="9" t="inlineStr">
-        <is>
-          <t>~-0.01%</t>
-        </is>
+      <c r="P2" s="6" t="n">
+        <v>-491.94</v>
+      </c>
+      <c r="Q2" s="9" t="n">
+        <v>-0.25</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -14127,7 +14129,7 @@
       </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
-          <t>#31ID Price&gt;SMA50+EMA20&lt;EMA50+Close&lt;Open</t>
+          <t>#31ID Price&gt;SMA50+EMA20&lt;EMA50+Close&lt;Open | Expiry 6h</t>
         </is>
       </c>
     </row>
@@ -14484,12 +14486,12 @@
       <c r="O6" s="4" t="n">
         <v>10.44</v>
       </c>
-      <c r="P6" s="9" t="inlineStr">
+      <c r="P6" s="10" t="inlineStr">
         <is>
           <t>~1,210.76 (unrealized)</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="Q6" s="10" t="inlineStr">
         <is>
           <t>~+2.34%</t>
         </is>
@@ -14581,12 +14583,12 @@
       <c r="O7" s="4" t="n">
         <v>10.42</v>
       </c>
-      <c r="P7" s="9" t="inlineStr">
+      <c r="P7" s="10" t="inlineStr">
         <is>
           <t>~-111.80 (unrealized)</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="10" t="inlineStr">
         <is>
           <t>~-0.19%</t>
         </is>
@@ -14678,12 +14680,12 @@
       <c r="O8" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="P8" s="9" t="inlineStr">
+      <c r="P8" s="10" t="inlineStr">
         <is>
           <t>~-131.66 (unrealized)</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
+      <c r="Q8" s="10" t="inlineStr">
         <is>
           <t>~-0.23%</t>
         </is>
@@ -14775,12 +14777,12 @@
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
-      <c r="P9" s="9" t="inlineStr">
+      <c r="P9" s="10" t="inlineStr">
         <is>
           <t>~52.24 (unrealized)</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
+      <c r="Q9" s="10" t="inlineStr">
         <is>
           <t>~+0.12%</t>
         </is>
@@ -14847,16 +14849,16 @@
           <t>SWING_1d</t>
         </is>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="11" t="n">
         <v>0.3393</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I10" s="12" t="n">
         <v>0.3315</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J10" s="12" t="n">
         <v>0.3518</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -14872,12 +14874,12 @@
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
-      <c r="P10" s="9" t="inlineStr">
+      <c r="P10" s="10" t="inlineStr">
         <is>
           <t>~-37.99 (unrealized)</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="10" t="inlineStr">
         <is>
           <t>~-0.82%</t>
         </is>
@@ -15043,16 +15045,16 @@
           <t>INTRADAY_1h</t>
         </is>
       </c>
-      <c r="G12" s="10" t="n">
+      <c r="G12" s="11" t="n">
         <v>0.083828</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>50000</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="12" t="n">
         <v>0.085341</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="J12" s="12" t="n">
         <v>0.08155800000000001</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -15374,7 +15376,7 @@
       <c r="P15" s="5" t="n">
         <v>273.16</v>
       </c>
-      <c r="Q15" s="12" t="n">
+      <c r="Q15" s="13" t="n">
         <v>0.52</v>
       </c>
       <c r="R15" s="2" t="inlineStr">
@@ -15736,16 +15738,16 @@
           <t>SWING_1d</t>
         </is>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="11" t="n">
         <v>0.3349</v>
       </c>
       <c r="H19" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="I19" s="11" t="n">
+      <c r="I19" s="12" t="n">
         <v>0.3272</v>
       </c>
-      <c r="J19" s="11" t="n">
+      <c r="J19" s="12" t="n">
         <v>0.3473</v>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -15770,7 +15772,7 @@
       <c r="P19" s="5" t="n">
         <v>24.96</v>
       </c>
-      <c r="Q19" s="12" t="n">
+      <c r="Q19" s="13" t="n">
         <v>0.75</v>
       </c>
       <c r="R19" s="2" t="inlineStr">
@@ -16265,7 +16267,7 @@
       <c r="P24" s="5" t="n">
         <v>332.63</v>
       </c>
-      <c r="Q24" s="12" t="n">
+      <c r="Q24" s="13" t="n">
         <v>0.66</v>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -16364,7 +16366,7 @@
       <c r="P25" s="5" t="n">
         <v>181.12</v>
       </c>
-      <c r="Q25" s="12" t="n">
+      <c r="Q25" s="13" t="n">
         <v>0.28</v>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -16463,7 +16465,7 @@
       <c r="P26" s="5" t="n">
         <v>65.36</v>
       </c>
-      <c r="Q26" s="12" t="n">
+      <c r="Q26" s="13" t="n">
         <v>0.13</v>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -16661,7 +16663,7 @@
       <c r="P28" s="5" t="n">
         <v>352.6</v>
       </c>
-      <c r="Q28" s="12" t="n">
+      <c r="Q28" s="13" t="n">
         <v>0.34</v>
       </c>
       <c r="R28" s="2" t="inlineStr">
@@ -16958,7 +16960,7 @@
       <c r="P31" s="5" t="n">
         <v>284.17</v>
       </c>
-      <c r="Q31" s="12" t="n">
+      <c r="Q31" s="13" t="n">
         <v>0.57</v>
       </c>
       <c r="R31" s="2" t="inlineStr">
@@ -17156,7 +17158,7 @@
       <c r="P33" s="5" t="n">
         <v>183.99</v>
       </c>
-      <c r="Q33" s="12" t="n">
+      <c r="Q33" s="13" t="n">
         <v>0.38</v>
       </c>
       <c r="R33" s="2" t="inlineStr">
@@ -17255,7 +17257,7 @@
       <c r="P34" s="6" t="n">
         <v>-479</v>
       </c>
-      <c r="Q34" s="13" t="n">
+      <c r="Q34" s="9" t="n">
         <v>-0.96</v>
       </c>
       <c r="R34" s="2" t="inlineStr">
@@ -17320,16 +17322,16 @@
           <t>SWING_1d</t>
         </is>
       </c>
-      <c r="G35" s="10" t="n">
+      <c r="G35" s="11" t="n">
         <v>0.3462</v>
       </c>
       <c r="H35" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="I35" s="11" t="n">
+      <c r="I35" s="12" t="n">
         <v>0.3382</v>
       </c>
-      <c r="J35" s="11" t="n">
+      <c r="J35" s="12" t="n">
         <v>0.3589</v>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -17453,7 +17455,7 @@
       <c r="P36" s="5" t="n">
         <v>373.92</v>
       </c>
-      <c r="Q36" s="12" t="n">
+      <c r="Q36" s="13" t="n">
         <v>0.76</v>
       </c>
       <c r="R36" s="2" t="inlineStr">
@@ -17552,7 +17554,7 @@
       <c r="P37" s="5" t="n">
         <v>35.91</v>
       </c>
-      <c r="Q37" s="12" t="n">
+      <c r="Q37" s="13" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="R37" s="2" t="inlineStr">
@@ -17651,7 +17653,7 @@
       <c r="P38" s="6" t="n">
         <v>-311.52</v>
       </c>
-      <c r="Q38" s="13" t="n">
+      <c r="Q38" s="9" t="n">
         <v>-0.63</v>
       </c>
       <c r="R38" s="2" t="inlineStr">
@@ -17750,7 +17752,7 @@
       <c r="P39" s="6" t="n">
         <v>-448.74</v>
       </c>
-      <c r="Q39" s="13" t="n">
+      <c r="Q39" s="9" t="n">
         <v>-0.87</v>
       </c>
       <c r="R39" s="2" t="inlineStr">
@@ -18112,16 +18114,16 @@
           <t>SWING_1d</t>
         </is>
       </c>
-      <c r="G43" s="10" t="n">
+      <c r="G43" s="11" t="n">
         <v>0.332</v>
       </c>
       <c r="H43" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="I43" s="11" t="n">
+      <c r="I43" s="12" t="n">
         <v>0.3244</v>
       </c>
-      <c r="J43" s="11" t="n">
+      <c r="J43" s="12" t="n">
         <v>0.3442</v>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -18344,7 +18346,7 @@
       <c r="P45" s="6" t="n">
         <v>-141.68</v>
       </c>
-      <c r="Q45" s="13" t="n">
+      <c r="Q45" s="9" t="n">
         <v>-0.28</v>
       </c>
       <c r="R45" s="2" t="inlineStr">
@@ -18443,7 +18445,7 @@
       <c r="P46" s="6" t="n">
         <v>-126.33</v>
       </c>
-      <c r="Q46" s="13" t="n">
+      <c r="Q46" s="9" t="n">
         <v>-0.25</v>
       </c>
       <c r="R46" s="2" t="inlineStr">
@@ -18641,7 +18643,7 @@
       <c r="P48" s="5" t="n">
         <v>19.63</v>
       </c>
-      <c r="Q48" s="12" t="n">
+      <c r="Q48" s="13" t="n">
         <v>0.04</v>
       </c>
       <c r="R48" s="2" t="inlineStr">
@@ -18706,16 +18708,16 @@
           <t>SWING_1d</t>
         </is>
       </c>
-      <c r="G49" s="10" t="n">
+      <c r="G49" s="11" t="n">
         <v>0.331</v>
       </c>
       <c r="H49" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="I49" s="11" t="n">
+      <c r="I49" s="12" t="n">
         <v>0.3241</v>
       </c>
-      <c r="J49" s="11" t="n">
+      <c r="J49" s="12" t="n">
         <v>0.3439</v>
       </c>
       <c r="K49" s="3" t="inlineStr">
@@ -18740,7 +18742,7 @@
       <c r="P49" s="6" t="n">
         <v>-15.49</v>
       </c>
-      <c r="Q49" s="13" t="n">
+      <c r="Q49" s="9" t="n">
         <v>-0.47</v>
       </c>
       <c r="R49" s="2" t="inlineStr">
@@ -18938,7 +18940,7 @@
       <c r="P51" s="5" t="n">
         <v>194.6</v>
       </c>
-      <c r="Q51" s="12" t="n">
+      <c r="Q51" s="13" t="n">
         <v>0.4</v>
       </c>
       <c r="R51" s="2" t="inlineStr">
@@ -19037,7 +19039,7 @@
       <c r="P52" s="6" t="n">
         <v>-76.67</v>
       </c>
-      <c r="Q52" s="13" t="n">
+      <c r="Q52" s="9" t="n">
         <v>-0.16</v>
       </c>
       <c r="R52" s="2" t="inlineStr">
@@ -19136,7 +19138,7 @@
       <c r="P53" s="5" t="n">
         <v>95.48</v>
       </c>
-      <c r="Q53" s="12" t="n">
+      <c r="Q53" s="13" t="n">
         <v>0.19</v>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -19235,7 +19237,7 @@
       <c r="P54" s="5" t="n">
         <v>440.05</v>
       </c>
-      <c r="Q54" s="12" t="n">
+      <c r="Q54" s="13" t="n">
         <v>0.86</v>
       </c>
       <c r="R54" s="2" t="inlineStr">
@@ -19300,16 +19302,16 @@
           <t>SWING_1d</t>
         </is>
       </c>
-      <c r="G55" s="10" t="n">
+      <c r="G55" s="11" t="n">
         <v>0.3281</v>
       </c>
       <c r="H55" s="4" t="n">
         <v>10000</v>
       </c>
-      <c r="I55" s="11" t="n">
+      <c r="I55" s="12" t="n">
         <v>0.3215</v>
       </c>
-      <c r="J55" s="11" t="n">
+      <c r="J55" s="12" t="n">
         <v>0.3412</v>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -19334,7 +19336,7 @@
       <c r="P55" s="5" t="n">
         <v>9.48</v>
       </c>
-      <c r="Q55" s="12" t="n">
+      <c r="Q55" s="13" t="n">
         <v>0.29</v>
       </c>
       <c r="R55" s="2" t="inlineStr">
@@ -20027,7 +20029,7 @@
       <c r="P62" s="5" t="n">
         <v>742.39</v>
       </c>
-      <c r="Q62" s="12" t="n">
+      <c r="Q62" s="13" t="n">
         <v>0.87</v>
       </c>
       <c r="R62" s="2" t="inlineStr">
@@ -20126,7 +20128,7 @@
       <c r="P63" s="5" t="n">
         <v>787.15</v>
       </c>
-      <c r="Q63" s="12" t="n">
+      <c r="Q63" s="13" t="n">
         <v>0.87</v>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -20225,7 +20227,7 @@
       <c r="P64" s="5" t="n">
         <v>679.01</v>
       </c>
-      <c r="Q64" s="12" t="n">
+      <c r="Q64" s="13" t="n">
         <v>0.76</v>
       </c>
       <c r="R64" s="2" t="inlineStr">
@@ -20324,7 +20326,7 @@
       <c r="P65" s="5" t="n">
         <v>787.02</v>
       </c>
-      <c r="Q65" s="12" t="n">
+      <c r="Q65" s="13" t="n">
         <v>0.86</v>
       </c>
       <c r="R65" s="2" t="inlineStr">
@@ -20423,7 +20425,7 @@
       <c r="P66" s="5" t="n">
         <v>298.29</v>
       </c>
-      <c r="Q66" s="12" t="n">
+      <c r="Q66" s="13" t="n">
         <v>0.32</v>
       </c>
       <c r="R66" s="2" t="inlineStr">
@@ -20518,7 +20520,7 @@
       <c r="P67" s="5" t="n">
         <v>298</v>
       </c>
-      <c r="Q67" s="12" t="n">
+      <c r="Q67" s="13" t="n">
         <v>0.32</v>
       </c>
       <c r="R67" s="2" t="inlineStr">
@@ -20613,7 +20615,7 @@
       <c r="P68" s="6" t="n">
         <v>-391.38</v>
       </c>
-      <c r="Q68" s="13" t="n">
+      <c r="Q68" s="9" t="n">
         <v>-0.41</v>
       </c>
       <c r="R68" s="2" t="inlineStr">
@@ -20699,7 +20701,7 @@
           <t>19:00:00 IST</t>
         </is>
       </c>
-      <c r="N69" s="10" t="n">
+      <c r="N69" s="11" t="n">
         <v>-0.92</v>
       </c>
       <c r="O69" s="4" t="n">
@@ -20708,7 +20710,7 @@
       <c r="P69" s="6" t="n">
         <v>-20</v>
       </c>
-      <c r="Q69" s="13" t="n">
+      <c r="Q69" s="9" t="n">
         <v>-0.02</v>
       </c>
       <c r="R69" s="2" t="inlineStr">
@@ -21042,18 +21044,18 @@
       <c r="L73" s="15" t="inlineStr"/>
       <c r="M73" s="14" t="inlineStr"/>
       <c r="N73" s="17" t="n">
-        <v>18523.39</v>
+        <v>18071.27</v>
       </c>
       <c r="O73" s="17" t="n">
-        <v>3592.33</v>
+        <v>3632.15</v>
       </c>
       <c r="P73" s="18" t="n">
-        <v>14931.06</v>
+        <v>14439.12</v>
       </c>
       <c r="Q73" s="16" t="inlineStr"/>
       <c r="R73" s="15" t="inlineStr">
         <is>
-          <t>71 trades (65 closed / 6 open)</t>
+          <t>71 trades (66 closed / 5 open)</t>
         </is>
       </c>
       <c r="S73" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
v5.12 scan 2026-09-18 20:48 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14481,19 +14481,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>1221.2</v>
+        <v>1669.92</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>~1,210.76 (unrealized)</t>
+          <t>~1,659.48 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
         <is>
-          <t>~+2.34%</t>
+          <t>~+3.20%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -14578,19 +14578,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="4" t="n">
-        <v>-101.38</v>
+        <v>-49.32</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.42</v>
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>~-111.80 (unrealized)</t>
+          <t>~-59.74 (unrealized)</t>
         </is>
       </c>
       <c r="Q7" s="10" t="inlineStr">
         <is>
-          <t>~-0.19%</t>
+          <t>~-0.09%</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -14675,19 +14675,19 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="4" t="n">
-        <v>-121.16</v>
+        <v>-838.8</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.5</v>
       </c>
       <c r="P8" s="10" t="inlineStr">
         <is>
-          <t>~-131.66 (unrealized)</t>
+          <t>~-849.30 (unrealized)</t>
         </is>
       </c>
       <c r="Q8" s="10" t="inlineStr">
         <is>
-          <t>~-0.23%</t>
+          <t>~-1.60%</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -14772,19 +14772,19 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="4" t="n">
-        <v>62.7</v>
+        <v>-369.93</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>~52.24 (unrealized)</t>
+          <t>~-380.39 (unrealized)</t>
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr">
         <is>
-          <t>~+0.12%</t>
+          <t>~-0.71%</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -14869,19 +14869,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-27.81</v>
+        <v>-7.82</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="10" t="inlineStr">
         <is>
-          <t>~-37.99 (unrealized)</t>
+          <t>~-18.00 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr">
         <is>
-          <t>~-0.82%</t>
+          <t>~-0.23%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-18 21:45 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14869,19 +14869,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-7.82</v>
+        <v>-8.369999999999999</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="10" t="inlineStr">
         <is>
-          <t>~-18.00 (unrealized)</t>
+          <t>~-18.55 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr">
         <is>
-          <t>~-0.23%</t>
+          <t>~-0.25%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
v5.12 scan 2026-09-18 22:46 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14869,19 +14869,19 @@
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="4" t="n">
-        <v>-8.369999999999999</v>
+        <v>-9.4</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
       <c r="P10" s="10" t="inlineStr">
         <is>
-          <t>~-18.55 (unrealized)</t>
+          <t>~-19.58 (unrealized)</t>
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr">
         <is>
-          <t>~-0.25%</t>
+          <t>~-0.28%</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
live pnl 2026-09-19 13:19 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -2323,17 +2323,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>#1SW TRX-USD LONG</t>
+          <t>#1ID DOGE-USD SHORT</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>TRX-USD</t>
+          <t>DOGE-USD</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2343,46 +2343,46 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>66.67</v>
+        <v>50.67</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>51.86</v>
+        <v>31.42</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="N27" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>-27.64</v>
+        <v>-88.45</v>
       </c>
       <c r="P27" s="4" t="n">
-        <v>40.12</v>
+        <v>12.57</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>-67.76000000000001</v>
+        <v>-101.02</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>-16.94</v>
+        <v>-101.02</v>
       </c>
     </row>
     <row r="28">
@@ -2391,17 +2391,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>#1ID DOGE-USD SHORT</t>
+          <t>#1SW TRX-USD LONG</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>DOGE-USD</t>
+          <t>TRX-USD</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2411,46 +2411,46 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>50.67</v>
+        <v>66.67</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>31.42</v>
+        <v>51.86</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>-88.45</v>
+        <v>-52.01</v>
       </c>
       <c r="P28" s="4" t="n">
-        <v>12.57</v>
+        <v>50.3</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>-101.02</v>
+        <v>-102.31</v>
       </c>
       <c r="R28" s="4" t="n">
-        <v>-101.02</v>
+        <v>-20.46</v>
       </c>
     </row>
     <row r="29">
@@ -14866,27 +14866,29 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="L10" s="2" t="n">
+        <v>0.3369</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19 18:49:29 IST</t>
+        </is>
+      </c>
       <c r="N10" s="4" t="n">
-        <v>-9.4</v>
+        <v>-24.37</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10.18</v>
       </c>
-      <c r="P10" s="10" t="inlineStr">
-        <is>
-          <t>~-19.58 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q10" s="10" t="inlineStr">
-        <is>
-          <t>~-0.28%</t>
-        </is>
+      <c r="P10" s="6" t="n">
+        <v>-34.55</v>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>-1.02</v>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -14911,7 +14913,7 @@
       </c>
       <c r="W10" s="3" t="inlineStr">
         <is>
-          <t>#1SW EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
+          <t>#1SW EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1% | Expiry 5d</t>
         </is>
       </c>
     </row>
@@ -21044,18 +21046,18 @@
       <c r="L73" s="15" t="inlineStr"/>
       <c r="M73" s="14" t="inlineStr"/>
       <c r="N73" s="17" t="n">
-        <v>18071.27</v>
+        <v>18046.9</v>
       </c>
       <c r="O73" s="17" t="n">
-        <v>3632.15</v>
+        <v>3642.33</v>
       </c>
       <c r="P73" s="18" t="n">
-        <v>14439.12</v>
+        <v>14404.57</v>
       </c>
       <c r="Q73" s="16" t="inlineStr"/>
       <c r="R73" s="15" t="inlineStr">
         <is>
-          <t>71 trades (66 closed / 5 open)</t>
+          <t>71 trades (67 closed / 4 open)</t>
         </is>
       </c>
       <c r="S73" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
live pnl 2026-09-20 00:01 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -2255,66 +2255,66 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>#4SW XLP LONG</t>
+          <t>#1ID DOGE-USD SHORT</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>SWING_1d</t>
+          <t>INTRADAY_1h</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>DOGE-USD</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CRYPTO</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>EMA20&lt;EMA50+Range&lt;1%</t>
+          <t>Price&gt;SMA20+RSI&lt;45</t>
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>61.78</v>
+        <v>50.67</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>70.52</v>
+        <v>31.42</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="K26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="4" t="n">
-        <v>0</v>
+        <v>-88.45</v>
       </c>
       <c r="P26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="4" t="n">
-        <v>0</v>
+        <v>12.57</v>
+      </c>
+      <c r="Q26" s="6" t="n">
+        <v>-101.02</v>
       </c>
       <c r="R26" s="4" t="n">
-        <v>0</v>
+        <v>-101.02</v>
       </c>
     </row>
     <row r="27">
@@ -2323,17 +2323,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>#1ID DOGE-USD SHORT</t>
+          <t>#1SW TRX-USD LONG</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>INTRADAY_1h</t>
+          <t>SWING_1d</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>DOGE-USD</t>
+          <t>TRX-USD</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2343,46 +2343,46 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA20+RSI&lt;45</t>
+          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H27" s="4" t="n">
-        <v>50.67</v>
+        <v>66.67</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>31.42</v>
+        <v>51.86</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O27" s="4" t="n">
-        <v>-88.45</v>
+        <v>-52.01</v>
       </c>
       <c r="P27" s="4" t="n">
-        <v>12.57</v>
+        <v>50.3</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>-101.02</v>
+        <v>-102.31</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>-101.02</v>
+        <v>-20.46</v>
       </c>
     </row>
     <row r="28">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>#1SW TRX-USD LONG</t>
+          <t>#5SW XLP LONG</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>TRX-USD</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>CRYPTO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2416,41 +2416,41 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>EMA9&gt;EMA20+Price&gt;SMA50+Range&lt;1%</t>
+          <t>Range&lt;1%+SMA20&lt;EMA20</t>
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>66.67</v>
+        <v>58.26</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>51.86</v>
+        <v>67.47</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="O28" s="4" t="n">
-        <v>-52.01</v>
+        <v>-149.74</v>
       </c>
       <c r="P28" s="4" t="n">
-        <v>50.3</v>
+        <v>20.27</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>-102.31</v>
+        <v>-170.01</v>
       </c>
       <c r="R28" s="4" t="n">
-        <v>-20.46</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="29">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>#5SW XLP LONG</t>
+          <t>#4SW XLP LONG</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2484,41 +2484,41 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Range&lt;1%+SMA20&lt;EMA20</t>
+          <t>EMA20&lt;EMA50+Range&lt;1%</t>
         </is>
       </c>
       <c r="H29" s="4" t="n">
-        <v>58.26</v>
+        <v>61.78</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>67.47</v>
+        <v>70.52</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O29" s="4" t="n">
-        <v>-149.74</v>
+        <v>-375.12</v>
       </c>
       <c r="P29" s="4" t="n">
-        <v>20.27</v>
+        <v>10.46</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>-170.01</v>
+        <v>-385.58</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>-85</v>
+        <v>-385.58</v>
       </c>
     </row>
     <row r="30">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>#3SW XLC LONG</t>
+          <t>#31SW QQQ LONG</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2620,20 +2620,20 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;EMA9+Range&lt;1%</t>
+          <t>Price&gt;SMA50+2Red</t>
         </is>
       </c>
       <c r="H31" s="4" t="n">
-        <v>53.98</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>68.92</v>
+        <v>48.57</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2645,16 +2645,16 @@
         <v>0</v>
       </c>
       <c r="O31" s="4" t="n">
-        <v>-750.65</v>
+        <v>-865.8099999999999</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>10.32</v>
+        <v>10.46</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>-760.97</v>
+        <v>-876.27</v>
       </c>
     </row>
     <row r="32">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>#31SW QQQ LONG</t>
+          <t>#5SW KBE LONG</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>KBE</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2688,14 +2688,14 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Price&gt;SMA50+2Red</t>
+          <t>EMA9&lt;EMA50+Price&gt;EMA50</t>
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>65.29000000000001</v>
+        <v>50.67</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>48.57</v>
+        <v>17.55</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1</v>
@@ -2713,16 +2713,16 @@
         <v>0</v>
       </c>
       <c r="O32" s="4" t="n">
-        <v>-865.8099999999999</v>
+        <v>-1039.2</v>
       </c>
       <c r="P32" s="4" t="n">
-        <v>10.46</v>
+        <v>10.29</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>-876.27</v>
+        <v>-1049.49</v>
       </c>
       <c r="R32" s="4" t="n">
-        <v>-876.27</v>
+        <v>-1049.49</v>
       </c>
     </row>
     <row r="33">
@@ -2769,28 +2769,28 @@
         <v>6</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>20</v>
+        <v>16.7</v>
       </c>
       <c r="O33" s="4" t="n">
-        <v>-982.38</v>
+        <v>-1036.91</v>
       </c>
       <c r="P33" s="4" t="n">
-        <v>50.18</v>
+        <v>60.6</v>
       </c>
       <c r="Q33" s="6" t="n">
-        <v>-1032.56</v>
+        <v>-1097.51</v>
       </c>
       <c r="R33" s="4" t="n">
-        <v>-206.51</v>
+        <v>-182.92</v>
       </c>
     </row>
     <row r="34">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>#5SW KBE LONG</t>
+          <t>#3SW XLC LONG</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>KBE</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2824,17 +2824,17 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>EMA9&lt;EMA50+Price&gt;EMA50</t>
+          <t>Price&gt;EMA9+Range&lt;1%</t>
         </is>
       </c>
       <c r="H34" s="4" t="n">
-        <v>50.67</v>
+        <v>53.98</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>17.55</v>
+        <v>68.92</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2843,22 +2843,22 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O34" s="4" t="n">
-        <v>-1039.2</v>
+        <v>-1594.61</v>
       </c>
       <c r="P34" s="4" t="n">
-        <v>10.29</v>
+        <v>20.82</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>-1049.49</v>
+        <v>-1615.43</v>
       </c>
       <c r="R34" s="4" t="n">
-        <v>-1049.49</v>
+        <v>-807.72</v>
       </c>
     </row>
     <row r="35">
@@ -14575,27 +14575,29 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="L7" s="2" t="n">
+        <v>379.99</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19 05:30:00 IST</t>
+        </is>
+      </c>
       <c r="N7" s="4" t="n">
-        <v>-49.32</v>
+        <v>-54.53</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>10.42</v>
       </c>
-      <c r="P7" s="10" t="inlineStr">
-        <is>
-          <t>~-59.74 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q7" s="10" t="inlineStr">
-        <is>
-          <t>~-0.09%</t>
-        </is>
+      <c r="P7" s="6" t="n">
+        <v>-64.95</v>
+      </c>
+      <c r="Q7" s="9" t="n">
+        <v>-0.12</v>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -14620,7 +14622,7 @@
       </c>
       <c r="W7" s="3" t="inlineStr">
         <is>
-          <t>#4SW EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1%</t>
+          <t>#4SW EMA9&gt;EMA20+Price&gt;SMA20+Range&lt;1% | Expiry 5d</t>
         </is>
       </c>
     </row>
@@ -14672,27 +14674,29 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="L8" s="2" t="n">
+        <v>110.8</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19 05:30:00 IST</t>
+        </is>
+      </c>
       <c r="N8" s="4" t="n">
-        <v>-838.8</v>
+        <v>-843.96</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="P8" s="10" t="inlineStr">
-        <is>
-          <t>~-849.30 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q8" s="10" t="inlineStr">
-        <is>
-          <t>~-1.60%</t>
-        </is>
+      <c r="P8" s="6" t="n">
+        <v>-854.46</v>
+      </c>
+      <c r="Q8" s="6" t="n">
+        <v>-1.63</v>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -14717,7 +14721,7 @@
       </c>
       <c r="W8" s="3" t="inlineStr">
         <is>
-          <t>#3SW Price&gt;EMA9+Range&lt;1%</t>
+          <t>#3SW Price&gt;EMA9+Range&lt;1% | Expiry 5d</t>
         </is>
       </c>
     </row>
@@ -14769,27 +14773,29 @@
           <t>5</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="L9" s="2" t="n">
+        <v>82.79000000000001</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19 05:30:00 IST</t>
+        </is>
+      </c>
       <c r="N9" s="4" t="n">
-        <v>-369.93</v>
+        <v>-375.12</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>10.46</v>
       </c>
-      <c r="P9" s="10" t="inlineStr">
-        <is>
-          <t>~-380.39 (unrealized)</t>
-        </is>
-      </c>
-      <c r="Q9" s="10" t="inlineStr">
-        <is>
-          <t>~-0.71%</t>
-        </is>
+      <c r="P9" s="6" t="n">
+        <v>-385.58</v>
+      </c>
+      <c r="Q9" s="9" t="n">
+        <v>-0.74</v>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -14814,7 +14820,7 @@
       </c>
       <c r="W9" s="3" t="inlineStr">
         <is>
-          <t>#4SW EMA20&lt;EMA50+Range&lt;1%</t>
+          <t>#4SW EMA20&lt;EMA50+Range&lt;1% | Expiry 5d</t>
         </is>
       </c>
     </row>
@@ -21046,18 +21052,18 @@
       <c r="L73" s="15" t="inlineStr"/>
       <c r="M73" s="14" t="inlineStr"/>
       <c r="N73" s="17" t="n">
-        <v>18046.9</v>
+        <v>16773.29</v>
       </c>
       <c r="O73" s="17" t="n">
-        <v>3642.33</v>
+        <v>3673.71</v>
       </c>
       <c r="P73" s="18" t="n">
-        <v>14404.57</v>
+        <v>13099.58</v>
       </c>
       <c r="Q73" s="16" t="inlineStr"/>
       <c r="R73" s="15" t="inlineStr">
         <is>
-          <t>71 trades (67 closed / 4 open)</t>
+          <t>71 trades (70 closed / 1 open)</t>
         </is>
       </c>
       <c r="S73" s="15" t="inlineStr"/>

</xml_diff>

<commit_message>
v5.12 scan 2026-09-21 05:17 UTC
</commit_message>
<xml_diff>
--- a/logs/strategy_report.xlsx
+++ b/logs/strategy_report.xlsx
@@ -14481,19 +14481,19 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="4" t="n">
-        <v>1669.92</v>
+        <v>1658.56</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>10.44</v>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>~1,659.48 (unrealized)</t>
+          <t>~1,648.12 (unrealized)</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
         <is>
-          <t>~+3.20%</t>
+          <t>~+3.18%</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">

</xml_diff>